<commit_message>
Préparation au deploiement des MAJ
</commit_message>
<xml_diff>
--- a/imports/EtatPaiement.xlsx
+++ b/imports/EtatPaiement.xlsx
@@ -10,6 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">A!$A$1:$M$233</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">A!$A$1:$M$233</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -21,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
   <si>
-    <t>matricule</t>
+    <t>Matricule</t>
   </si>
   <si>
     <t>IDannee</t>
@@ -57,7 +58,7 @@
     <t>date_paie</t>
   </si>
   <si>
-    <t>id_etat_paie</t>
+    <t>IDEtat</t>
   </si>
   <si>
     <t>24527</t>
@@ -10819,134 +10820,134 @@
       </c>
     </row>
     <row r="234" ht="15" customHeight="1">
-      <c r="G234" s="5"/>
-      <c r="H234" s="5"/>
+      <c r="G234"/>
+      <c r="H234"/>
     </row>
     <row r="235" ht="15" customHeight="1">
-      <c r="G235" s="5"/>
-      <c r="H235" s="5"/>
+      <c r="G235"/>
+      <c r="H235"/>
     </row>
     <row r="236" ht="15" customHeight="1">
-      <c r="G236" s="5"/>
-      <c r="H236" s="5"/>
+      <c r="G236"/>
+      <c r="H236"/>
     </row>
     <row r="237" ht="15" customHeight="1">
-      <c r="G237" s="5"/>
-      <c r="H237" s="5"/>
+      <c r="G237"/>
+      <c r="H237"/>
     </row>
     <row r="238" ht="15" customHeight="1">
-      <c r="G238" s="5"/>
-      <c r="H238" s="5"/>
+      <c r="G238"/>
+      <c r="H238"/>
     </row>
     <row r="239" ht="15" customHeight="1">
-      <c r="G239" s="5"/>
-      <c r="H239" s="5"/>
+      <c r="G239"/>
+      <c r="H239"/>
     </row>
     <row r="240" ht="15" customHeight="1">
-      <c r="G240" s="5"/>
-      <c r="H240" s="5"/>
+      <c r="G240"/>
+      <c r="H240"/>
     </row>
     <row r="241" ht="15" customHeight="1">
-      <c r="G241" s="5"/>
-      <c r="H241" s="5"/>
+      <c r="G241"/>
+      <c r="H241"/>
     </row>
     <row r="242" ht="15" customHeight="1">
-      <c r="G242" s="5"/>
-      <c r="H242" s="5"/>
+      <c r="G242"/>
+      <c r="H242"/>
     </row>
     <row r="243" ht="15" customHeight="1">
-      <c r="G243" s="5"/>
-      <c r="H243" s="5"/>
+      <c r="G243"/>
+      <c r="H243"/>
     </row>
     <row r="244" ht="15" customHeight="1">
-      <c r="H244" s="5"/>
+      <c r="H244"/>
     </row>
     <row r="245" ht="15" customHeight="1">
-      <c r="H245" s="5"/>
+      <c r="H245"/>
     </row>
     <row r="246" ht="15" customHeight="1">
-      <c r="H246" s="5"/>
+      <c r="H246"/>
     </row>
     <row r="247" ht="15" customHeight="1">
-      <c r="H247" s="5"/>
+      <c r="H247"/>
     </row>
     <row r="248" ht="15" customHeight="1">
-      <c r="H248" s="5"/>
+      <c r="H248"/>
     </row>
     <row r="249" ht="15" customHeight="1">
-      <c r="H249" s="5"/>
+      <c r="H249"/>
     </row>
     <row r="250" ht="15" customHeight="1">
-      <c r="H250" s="5"/>
+      <c r="H250"/>
     </row>
     <row r="251" ht="15" customHeight="1">
-      <c r="H251" s="5"/>
+      <c r="H251"/>
     </row>
     <row r="252" ht="15" customHeight="1">
-      <c r="H252" s="5"/>
+      <c r="H252"/>
     </row>
     <row r="253" ht="15" customHeight="1">
-      <c r="H253" s="5"/>
+      <c r="H253"/>
     </row>
     <row r="254" ht="15" customHeight="1">
-      <c r="H254" s="5"/>
+      <c r="H254"/>
     </row>
     <row r="255" ht="15" customHeight="1">
-      <c r="H255" s="5"/>
+      <c r="H255"/>
     </row>
     <row r="256" ht="15" customHeight="1">
-      <c r="H256" s="5"/>
+      <c r="H256"/>
     </row>
     <row r="257" ht="15" customHeight="1">
-      <c r="H257" s="5"/>
+      <c r="H257"/>
     </row>
     <row r="258" ht="15" customHeight="1">
-      <c r="H258" s="5"/>
+      <c r="H258"/>
     </row>
     <row r="259" ht="15" customHeight="1">
-      <c r="H259" s="5"/>
+      <c r="H259"/>
     </row>
     <row r="260" ht="15" customHeight="1">
-      <c r="H260" s="5"/>
+      <c r="H260"/>
     </row>
     <row r="261" ht="15" customHeight="1">
-      <c r="H261" s="5"/>
+      <c r="H261"/>
     </row>
     <row r="262" ht="15" customHeight="1">
-      <c r="H262" s="5"/>
+      <c r="H262"/>
     </row>
     <row r="263" ht="15" customHeight="1">
-      <c r="H263" s="5"/>
+      <c r="H263"/>
     </row>
     <row r="264" ht="15" customHeight="1">
-      <c r="H264" s="5"/>
+      <c r="H264"/>
     </row>
     <row r="265" ht="15" customHeight="1">
-      <c r="H265" s="5"/>
+      <c r="H265"/>
     </row>
     <row r="266" ht="15" customHeight="1">
-      <c r="H266" s="5"/>
+      <c r="H266"/>
     </row>
     <row r="267" ht="15" customHeight="1">
-      <c r="H267" s="5"/>
+      <c r="H267"/>
     </row>
     <row r="268" ht="15" customHeight="1">
-      <c r="H268" s="5"/>
+      <c r="H268"/>
     </row>
     <row r="269" ht="15" customHeight="1">
-      <c r="H269" s="5"/>
+      <c r="H269"/>
     </row>
     <row r="270" ht="15" customHeight="1">
-      <c r="H270" s="5"/>
+      <c r="H270"/>
     </row>
     <row r="271" ht="15" customHeight="1">
-      <c r="H271" s="5"/>
+      <c r="H271"/>
     </row>
     <row r="272" ht="15" customHeight="1">
-      <c r="H272" s="5"/>
+      <c r="H272"/>
     </row>
     <row r="273" ht="15" customHeight="1">
-      <c r="H273" s="5"/>
+      <c r="H273"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M233"/>

</xml_diff>